<commit_message>
fix: handle missing inventory without breaking plan responses
</commit_message>
<xml_diff>
--- a/examples/inventory.xlsx
+++ b/examples/inventory.xlsx
@@ -7,9 +7,11 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inventory" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$I$17</definedName>
+  </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -413,8 +415,19 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I12"/>
+  <dimension ref="A1:I17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="22" customWidth="1" min="8" max="8"/>
+    <col width="22" customWidth="1" min="9" max="9"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -470,7 +483,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>1000</v>
+        <v>42.6</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -479,14 +492,14 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="E2" t="n">
         <v>3000</v>
       </c>
       <c r="F2" t="n">
-        <v>0</v>
+        <v>1.5</v>
       </c>
       <c r="G2" t="n">
         <v>0</v>
@@ -509,7 +522,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>1000</v>
+        <v>18.75</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -518,14 +531,14 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="E3" t="n">
         <v>3000</v>
       </c>
       <c r="F3" t="n">
-        <v>0</v>
+        <v>2.15</v>
       </c>
       <c r="G3" t="n">
         <v>0</v>
@@ -548,7 +561,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>1000</v>
+        <v>91.3</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -557,14 +570,14 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-09-26</t>
         </is>
       </c>
       <c r="E4" t="n">
         <v>6100</v>
       </c>
       <c r="F4" t="n">
-        <v>0</v>
+        <v>2.8</v>
       </c>
       <c r="G4" t="n">
         <v>0</v>
@@ -587,7 +600,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>1000</v>
+        <v>138.7</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -596,14 +609,14 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="E5" t="n">
         <v>9000</v>
       </c>
       <c r="F5" t="n">
-        <v>0</v>
+        <v>3.45</v>
       </c>
       <c r="G5" t="n">
         <v>0</v>
@@ -626,7 +639,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>1000</v>
+        <v>106.4</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -635,14 +648,14 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="E6" t="n">
         <v>10000</v>
       </c>
       <c r="F6" t="n">
-        <v>0</v>
+        <v>4.1</v>
       </c>
       <c r="G6" t="n">
         <v>0</v>
@@ -665,7 +678,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>1000</v>
+        <v>37.8</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -674,14 +687,14 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="E7" t="n">
         <v>2000</v>
       </c>
       <c r="F7" t="n">
-        <v>0</v>
+        <v>4.75</v>
       </c>
       <c r="G7" t="n">
         <v>0</v>
@@ -704,7 +717,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>1000</v>
+        <v>24.6</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -713,14 +726,14 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="E8" t="n">
         <v>4000</v>
       </c>
       <c r="F8" t="n">
-        <v>0</v>
+        <v>5.4</v>
       </c>
       <c r="G8" t="n">
         <v>0</v>
@@ -743,7 +756,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>1000</v>
+        <v>44.2</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -752,14 +765,14 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="E9" t="n">
         <v>1800</v>
       </c>
       <c r="F9" t="n">
-        <v>0</v>
+        <v>6.05</v>
       </c>
       <c r="G9" t="n">
         <v>0</v>
@@ -782,7 +795,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>1000</v>
+        <v>23.9</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -791,14 +804,14 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="E10" t="n">
         <v>5000</v>
       </c>
       <c r="F10" t="n">
-        <v>0</v>
+        <v>6.7</v>
       </c>
       <c r="G10" t="n">
         <v>0</v>
@@ -821,7 +834,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>1000</v>
+        <v>12.8</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -830,14 +843,14 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-03</t>
         </is>
       </c>
       <c r="E11" t="n">
         <v>1000</v>
       </c>
       <c r="F11" t="n">
-        <v>0</v>
+        <v>7.35</v>
       </c>
       <c r="G11" t="n">
         <v>0</v>
@@ -860,7 +873,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>1000</v>
+        <v>72.34999999999999</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -869,14 +882,14 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="E12" t="n">
         <v>30000</v>
       </c>
       <c r="F12" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="G12" t="n">
         <v>0</v>
@@ -892,7 +905,203 @@
         </is>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>쌀</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>246.8</v>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>2026-12-18</t>
+        </is>
+      </c>
+      <c r="E13" t="n">
+        <v>2780</v>
+      </c>
+      <c r="F13" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="G13" t="n">
+        <v>0</v>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>ambient</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>잡곡</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>52.4</v>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>2026-12-03</t>
+        </is>
+      </c>
+      <c r="E14" t="n">
+        <v>4650</v>
+      </c>
+      <c r="F14" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="G14" t="n">
+        <v>0</v>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>ambient</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>된장</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>31.65</v>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>2026-11-03</t>
+        </is>
+      </c>
+      <c r="E15" t="n">
+        <v>5200</v>
+      </c>
+      <c r="F15" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="G15" t="n">
+        <v>0</v>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>refrigerated</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>미역</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>9.35</v>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>2027-01-17</t>
+        </is>
+      </c>
+      <c r="E16" t="n">
+        <v>14800</v>
+      </c>
+      <c r="F16" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="G16" t="n">
+        <v>0</v>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>ambient</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>콩나물</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>61.7</v>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="E17" t="n">
+        <v>1850</v>
+      </c>
+      <c r="F17" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="G17" t="n">
+        <v>0</v>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>refrigerated</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
+  <autoFilter ref="A1:I17"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>